<commit_message>
Add 42 containerised weapon systems; add Tier-C watch-list
Expands the registry from 27 to 69 systems, sourced from parallel deep
research and cross-checked against an independent ChatGPT deep-research
pass. New entries span directed-energy (THOR, DragonFire, Iron Beam,
Cheongwang, Kawasaki HEL, Rheinmetall/MBDA LWD, Epirus Leonidas),
C-UAS (Liteye C-AUDS, Diehl IRIS-T SLM, EDGE SKYSHIELD, VAMPIRE CASKET),
covert/strike launchers (CSDCS, Kara Atmaca, EREN, AReS, BlitzBox,
SLB-500M, Shahed-136, CM-401, Ruta Block 3), coastal (Saab RBS15 CDMS),
container-deployed autonomous vehicles (Seagull, Chaser, Speartooth,
XV Excalibur, BlueWhale) and modular architectures (IAI DIAMOND).

Each row carries a high/medium confidence flag and up to three cited
sources. Concept/programme-stage and overlapping candidates are held in
data/watchlist-candidates.csv rather than the main dataset. Photo fields
are left blank pending image sourcing.
</commit_message>
<xml_diff>
--- a/data/systems.xlsx
+++ b/data/systems.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W28"/>
+  <dimension ref="A1:W70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -819,8 +819,6 @@
           <t>LORA (missile) — Wikipedia</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -928,8 +926,6 @@
           <t>NAVDEX 2019: MBDA unveils the Self-Protection Integrated Mistral Module (SPIMM) for surface ship — EDR Magazine</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1037,8 +1033,6 @@
           <t>The Cube — EDGE Defence Ltd</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1136,10 +1130,6 @@
           <t>C-DOME: Maritime Application of the Combat-Proven Iron Dome — Rafael</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1247,8 +1237,6 @@
           <t>U.S. Navy Brings Offensive Capability To LCS With Mk 70 PDS — Naval News</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1346,10 +1334,6 @@
           <t>HUNTER 10 Long-Range Multi Role Loitering Munition — EDGE Group</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1457,8 +1441,6 @@
           <t>China's truck drone launcher hides airpower in civilian traffic — Asia Times</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1566,8 +1548,6 @@
           <t>Patria NEMO Container — 120 mm mortar system (product sheet)</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1675,8 +1655,6 @@
           <t>Naval Strike Missile (NSM) Coastal Defence System — Kongsberg</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1784,8 +1762,6 @@
           <t>U.S. Navy And Army Mk 70 PDS Stretch Their Wings — Naval News</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1893,8 +1869,6 @@
           <t>North Korea Debuts Rocket Launchers That Appear As Civilian Trucks — The War Zone</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1992,10 +1966,6 @@
           <t>If It Floats, It Fights: Containerised Naval Munitions — ESD</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2103,8 +2073,6 @@
           <t>Iran's Modern Q-Ship: A Threat from New Quarters — RUSI</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2212,8 +2180,6 @@
           <t>Shipping Container Launcher Packing 126 Kamikaze Drones — UAS Vision</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2311,10 +2277,6 @@
           <t>Mysterious Guided Rocket Launcher Disguised In A Shipping Container At Fort Bragg Identified — The War Zone</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2412,10 +2374,6 @@
           <t>CWS-A — Invariant Corp.</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2523,8 +2481,6 @@
           <t>Babcock and Frankenburg will build a containerized launch system for anti-drone missiles — Resilience Media</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2622,10 +2578,6 @@
           <t>If It Floats, It Fights: Containerised Naval Munitions — ESD</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2723,10 +2675,6 @@
           <t>Operation Spiderweb — Wikipedia</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2834,8 +2782,6 @@
           <t>Locust — AeroVironment</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2943,8 +2889,6 @@
           <t>Chinese Cargo Ship Packed Full Of Modular Missile Launchers Emerges — The War Zone</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3042,10 +2986,6 @@
           <t>Turkey just unveiled a 19.8-ton drone submarine built to launch FPV drone swarms, anti-ship missiles, torpedoes and mines while submerged — Autonocion.com</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3143,10 +3083,6 @@
           <t>Containerized Variant Of Navy's Drone-Swatting HELIOS Laser Being Pushed By Congress — The War Zone</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3254,8 +3190,6 @@
           <t>Hellfire Missile Launcher Tucked Inside A Container Rolled Out By Lockheed — The War Zone</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3353,10 +3287,6 @@
           <t>Hanwha Unveils Striker MUSV Family at Eurosatory 2026 — Naval News</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3464,8 +3394,3928 @@
           <t>Containerised Missile Launcher makes its debut at Eurosatory — Rheinmetall</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>csdcs</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CSDCS Container-Type Sea Defense Combat System</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CSDCS, containerized coastal defense system, China's Club-K</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CASIC (China Aerospace Science and Industry Corp)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2022-11-08</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>November 2022</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Unveiled at Airshow China (Zhuhai)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Missile launcher</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>A self-contained combat system built into a 20/40-ft container (~13m x 2.3m x 2.5m) with operator station, power and a quadruple launcher firing YJ-12E supersonic or YJ-18E subsonic anti-ship cruise missiles from ships, trucks or trains; China's openly-marketed Club-K analogue with broader missile compatibility.</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Distinct from the Zhong Da 79 arsenal-ship entry already in the list; this is the standalone containerized launcher product.</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>https://www.globaltimes.cn/page/202211/1279349.shtml</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>China debuts container-type missile launch system - Global Times</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>https://en.defence-ua.com/news/in_2022_china_unveiled_its_copy_of_russias_club_k_missile_system_now_it_threatens_us_navy-14827.html</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>China unveiled its copy of Russia's Club-K - Defense Express</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>https://www.vermilionchina.com/p/36-chinas-container-launched-cruise</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>China's Container-launched Cruise Missiles - Vermilion China</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>yj-18c</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>YJ-18C Container-Launched Cruise Missile</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>YJ-18C, container-launched YJ-18 land-attack variant</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CASC (China Aerospace Science and Technology Corp)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2019-03-01</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>March 2019</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>US intelligence-sourced reporting of container-launched variant</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Covert strike</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Concealed cargo</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Reported land-attack variant of the YJ-18 cruise missile (&gt;1,000 km, low-RCS) designed to fire from launchers built to look like standard ISO shipping containers on merchant-ship decks or trucks; conceptually a Chinese Club-K.</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Traces to a single 2019 US-intel report; missile never officially shown separately from the container concept.</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>https://freebeacon.com/national-security/china-building-long-range-cruise-missile-launched-from-ship-container/</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>China Building Cruise Missile Launched from Ship Container - Free Beacon</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/archives/archives-naval-defense/naval-defense-2019/china-is-building-long-range-cruise-missiles-launched-from-ship-containers</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>China building long-range cruise missiles from ship containers - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>https://www.scmp.com/news/china/military/article/3341929/will-new-chinas-yj-18c-missile-be-logistics-killer-us-navy</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Will China's YJ-18C missile be a logistics killer - SCMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ivan-papanin-kalibr-k</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Project 23550 Ivan Papanin Kalibr-K Container Module</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ivan Papanin containerized Kalibr, Project 23550 combat icebreaker</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Admiralty Shipyards / Morinformsystem-Agat lineage</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2021-10-15</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>October 2021</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Naval News detailed the containerized-bay design; lead ship commissioned Sept 2025</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Naval arsenal</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Modular deck launcher</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Purpose-built Arctic combat icebreaker/patrol ship with an open stern flex-bay designed to accept containerized Kalibr-K cruise-missile or Kh-35 anti-ship modules (up to 8 missiles); Russia's first near-operational Club-K-style warship fit.</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Missile module reportedly not yet installed at commissioning (only the 76mm gun fitted); deck pre-wired for retrofit.</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2021/10/russia-arctic-patrol-ship-cruise-missiles/</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Russia's Arctic Patrol Ships to Feature Cruise Missiles - Naval News</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/navy-news/2024/russian-navys-new-ivan-papanin-project-23550-combat-icebreaker-begins-sea-trials-with-kalibr-missiles</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Ivan Papanin begins sea trials with Kalibr - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>cm-300la</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Iran CM-300LA Land-Attack Container Launcher</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>CM-300LA, Container Missile-300 Land Attack</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Iranian defence industry (AIO/Shahid Bagheri lineage)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Shown at PARTNER 2025 exhibition (Belgrade)</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Covert strike</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>A three-round canister built to mimic a standard 20-ft ISO container on a civilian-style 6x6 truck, firing a subsonic (~300 km) sea-skimming land-attack cruise missile; onboard power, auto-leveling and shoot-and-scoot salvo capability.</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Reported by three trade outlets from the same unveiling; no TWZ/Naval News/Janes coverage yet.</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/army-news/2025/iran-presents-cm-300la-land-attack-container-launcher-firing-three-cruise-missiles-in-minutes</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Iran Presents CM-300LA Land-Attack Container Launcher - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>https://milivox.media/iran-cm300la-cruise-missile-container-launcher/</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Iran Unveils CM-300LA Containerized Cruise Missile Launcher - Milivox</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>shahed-136-container-launcher</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Iran Shahed-136 Tilting Container Drone Launcher</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Shahed-136 catapult-container system, Great Prophet 17 launcher</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>HESA / IRGC Aerospace Force</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2021-12-24</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>December 2021</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Unveiled during Great Prophet 17 exercise</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Loitering munition</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>A tilting truck-mounted container-like box holding up to five Shahed-136 loitering munitions, each rocket-boosted into flight; container form factor allows palletizing onto rail cars, ships or other vehicles.</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Well corroborated; distinct from later no-container pickup-truck launch method.</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>https://iranprimer.usip.org/blog/2021/dec/28/irgc-tests-ballistic-missiles-drones-war-game</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>IRGC Tests Ballistic Missiles, Drones in War Game - USIP</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>https://militarnyi.com/en/news/shahed-loitering-munition-received-the-capability-to-be-launched-from-a-vehicle/</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Shahed launched from a vehicle - Militarnyi</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>shahid-roudaki</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Iran Shahid Roudaki Twin Container Anti-Ship Launchers</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Shahid Roudaki forward-base ship container launchers, Qader/Ghadir deck launchers</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>IRGC Navy (converted from merchant Galaxy F)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2020-11-19</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>November 2020</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Commissioning ceremony reveal</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Naval arsenal</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Modular deck launcher</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Four twin box/container-style launchers (eight Qader/Ghadir anti-ship cruise missiles) bolted to the forward deck of a converted forward-base ship, alongside road-mobile radar.</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>H.I. Sutton flagged some displayed equipment may have been staged for the ceremony rather than integrated.</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>https://www.hisutton.com/Iranian-IRGC-Forward-Base-Shahid-Roudaki.html</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Iranian IRGC Forward Base Shahid Roudaki - Covert Shores</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>https://news.usni.org/2020/11/19/video-iran-inducts-new-special-operations-ship</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Iran Inducts New Special Operations Ship - USNI</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>hezbollah-container-launcher</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Hezbollah Container-Concealed Launcher Trucks</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Hezbollah closed-container hydraulic launcher, Paveh-351 container truck</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Hezbollah (Iranian-supplied)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Lebanon</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2022-11-01</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Documented doctrine; Nov 2022 Israeli strike on a Paveh container truck</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Covert / disguised</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Concealed cargo</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Hezbollah mounts Iranian-supplied rockets/cruise missiles on civilian trucks within closed containers that open hydraulically to erect and fire, dispersed in populated areas for survivability.</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Described launch method/doctrine (Alma Research) rather than one photographed named system; secondary confirmation thinner.</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>https://israel-alma.org/hezbollahs-heavy-rocket-array-medium-range-up-to-200-km-and-its-ballistic-missile-array-constitute-strategic-capabilities-of-the-organization/</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Hezbollah's heavy rocket array - Alma Research</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>https://israel-alma.org/iranian-paveh-cruise-missile-351-supplied-to-lebanese-hezbollah/</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Iranian Paveh Cruise Missile supplied to Hezbollah - Alma Research</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>hwasal-2-container</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>North Korea Hwasal-2 Container Cruise-Missile Launcher</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Hwasal-2 angled container launcher, Amnok-class corvette cruise-missile box</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>North Korean state defence industry</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>North Korea (DPRK)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2023-08-01</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>August 2023</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Naval version revealed on Amnok-class corvette; ground debut Oct 2021</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Strike missile</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Nuclear-capable land-attack cruise missile (~1,500-2,000 km) launched from an angled, box-like container rather than a VLS; seen in a 5-tube road-mobile launcher and an 8-tube aft-deck fit on the Amnok-class corvette.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Ambiguity over whether 'container' means a true ISO box or an inclined canister bank.</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Hwasal-2</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Hwasal-2 - Wikipedia</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2023/08/north-korea-new-cruise-missile-amnok-class-corvette/</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>North Korea reveals cruise missile-armed corvette - Naval News</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>dprk-harop-launcher</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>North Korea Harop-Type Loitering Munition Container Launcher</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DPRK Harop-clone container launcher, six-cell suicide-drone box</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>North Korean state defence industry</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>North Korea (DPRK)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2025-10-10</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>October 2025</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Displayed at Pyongyang parade (80th WPK anniversary)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Loitering munition</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>A 6x6 armored truck carrying two rows of three container-style launch cells for Harop-style kamikaze drones, marking a shift from 2024's bare-airframe reveal to fieldable launch hardware.</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Single-source detailed reporting; technical detail relies on analyst inference.</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/army-news/2025/north-korea-rolls-out-harop-type-loitering-munition-launcher-in-pyongyang-parade</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>North Korea rolls out Harop-type loitering munition launcher - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>https://militarnyi.com/en/news/north-korea-presents-launcher-for-copies-of-israeli-harop-kamikaze-drones/</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>North Korea Presents Launcher for Harop Copies - Militarnyi</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>thor-hpm</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>THOR</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Tactical High-power Operational Responder</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Air Force Research Laboratory (AFRL)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2019-06-01</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Development and swarm-defeat testing at Kirtland AFB</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>High-power microwave counter-swarm weapon stored in a standard 20-ft ISO container, C-130 transportable, set up in hours for airbase point defense against drone swarms.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Follow-on is Mjolnir (Leidos).</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>https://www.twz.com/thor-microwave-anti-drone-system-downs-swarms-in-test</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>THOR Microwave Anti-Drone System Downs Swarms - TWZ</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>https://www.airandspaceforces.com/air-forces-thor-drone-swarm-demo/</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>THOR Hammers Drone Swarm - Air &amp; Space Forces Magazine</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/THOR_(weapon)</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>THOR (weapon) - Wikipedia</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>mjolnir-hpm</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Mjolnir</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>THOR follow-on high-power microwave</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Leidos / Air Force Research Laboratory</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2021-03-01</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Development contract award</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Next-generation high-power microwave counter-swarm weapon derived from THOR, packaged in a transportable ISO container.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Container form-factor inherited from THOR.</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>https://afresearchlab.com/technology/directed-energy/</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>AFRL Directed Energy</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>https://www.leidos.com/insights/leidos-awarded-contract-develop-next-generation-high-power-microwave-weapon</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Leidos next-gen HPM weapon - Leidos</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>epirus-leonidas</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Epirus Leonidas (IFPC-HPM)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Leonidas, IFPC-HPM, Indirect Fire Protection Capability-High Power Microwave</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Epirus Inc.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2023-01-15</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>January 2023</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>US Army selection ($66.1M); prototypes delivered 2023-2024</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Solid-state GaN high-power microwave system that disables drone swarms; the base/IFPC-HPM unit fits inside a standard 20-ft container. Live-fire demo Aug 2025 downed 61 drones.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Only the base/IFPC-HPM version is containerized; Mobile/Pod/Expeditionary variants are not.</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>https://breakingdefense.com/2025/02/high-power-microwave-force-field-knocks-drone-swarms-from-sky/</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>HPM force field knocks drone swarms from sky - Breaking Defense</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>https://www.defensedaily.com/ifpc-hpm-prototype-deliveries-complete-epirus-eyes-engineering-tests-ahead-of-potential-deployment/army/</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>IFPC-HPM Prototype Deliveries Complete - Defense Daily</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>liteye-c-auds</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Liteye C-AUDS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>C-AUDS, Containerized Anti-UAS Defense System</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Liteye Systems (integrating UK AUDS tech)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2018-09-05</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>September 2018</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>USAF follow-on contract; production units delivered Dec 2018</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Air defense / C-UAS</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Integrates AUDS radar (Blighter), EO/IR tracker (Chess Dynamics) and RF-jamming effector (optional kinetic add-on) into a self-contained 20-ft ISO container for base and critical-infrastructure defense.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Base AUDS is vehicle/trailer-mounted; only the C-AUDS repackaging is a true container.</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>https://equipment.adsinc.com/</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Liteye C-AUDS product page - ADS</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>https://www.unmannedairspace.info/</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Blighter to supply C-UAS radar to Liteye - Unmanned Airspace</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>dzyne-blitzbox</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>DZYNE BlitzBox</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BlitzBox, Blitz drone container launcher</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>DZYNE Technologies</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Unveiled at SOF Week</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Loitering munition</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Concealed cargo</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>An ordinary-looking shipping container hiding a launch system for DZYNE's Blitz Group-1 expendable swarming drones; a 10-ft container holds 16 drones on 4 rail launchers, a 40-ft container up to 100.</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>TWZ direct interview with DZYNE program manager.</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>https://www.twz.com/</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>BlitzBox Packs 100 Weaponized Drones Into A Container - TWZ</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>https://www.slashgear.com/</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>A Container Full Of 100 Deadly Drones - SlashGear</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>dragonfire</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>DragonFire</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>DragonFire laser directed-energy weapon</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>MBDA UK / Leonardo UK / QinetiQ / Dstl</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2024-01-19</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>January 2024</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>First UK high-power live firing vs aerial targets (Hebrides Range)</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>50kW-class laser weapon whose land-trial unit is described as roughly the size of a TEU shipping container; £316m production contract (Nov 2025) to arm Royal Navy Type 45 destroyers by 2027.</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Shipboard-fitted version's exact housing less certain than the land-test container configuration.</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>https://www.naval-technology.com/news/dragonfire-uk-royal-navy-to-get-ships-with-laser-beams-by-2027/</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>DragonFire: Royal Navy laser by 2027 - Naval Technology</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>https://breakingdefense.com/2024/01/in-first-uk-test-fires-13-per-strike-dragonfire-laser-weapon-against-aerial-targets/</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>UK test fires DragonFire laser - Breaking Defense</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>rheinmetall-mbda-lwd</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Rheinmetall/MBDA Laser Weapon Demonstrator</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>LWD, 20kW naval laser demonstrator</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Rheinmetall + MBDA Deutschland</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2022-10-01</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>October 2022</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Installed on frigate Sachsen; sea trials 2022-2023</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>20kW-scalable laser demonstrator with turret and support equipment housed in a standard 20-ft container, craned onto the frigate Sachsen for a year of at-sea firing trials against drones and small boats.</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>In-service target ~2029.</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2025/10/rheinmetall-and-mbda-german-laser-weapon-system-close-to-market-readiness/</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>German laser weapon close to market readiness - Naval News</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>https://www.edrmagazine.eu/mbda-deutschland-provided-new-details-on-the-laser-weapon-demonstrator</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>MBDA Laser Weapon Demonstrator details - EDR Magazine</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>iron-beam</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Iron Beam</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Magen Or, Light Shield, Iron Beam 450</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Rafael Advanced Defense Systems (Elbit laser source)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>First operational unit delivered to IDF</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>100kW-class laser (ten fused 10kW fiber lasers) with a dome turret; beam-generation and cooling equipment described as housed in two 40-ft container-like modules, generally stationary but relocatable.</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>The 'two 40-ft container modules' phrasing recurs in secondary sources but primary ISO-container wording not verified.</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Iron_Beam</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Iron Beam - Wikipedia</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/army-news/2025/rafael-delivers-israels-first-operational-iron-beam-laser-shield-to-revolutionize-air-defense-era</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Rafael Delivers First Operational Iron Beam - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>silent-hunter</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Silent Hunter</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Shen Nu, Silent Hunter laser air-defence</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Poly Technologies</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2017-02-01</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>February 2017</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Unveiled at IDEX 2017; Saudi operational use vs Houthi drones</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>30-100kW-class anti-drone fiber laser; the mobile version is described as installed in a container towed by a 6x6 truck. Exported to the UAE/Saudi Arabia.</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Some sources describe it as separate truck-sized power and equipment units rather than a clear ISO box.</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Silent_Hunter_(laser_weapon)</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Silent Hunter (laser weapon) - Wikipedia</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>https://armyrecognition.com/news/army-news/army-news-2024/dsa-2024-chinese-company-poly-technologies-showcases-silent-hunter-laser-defense-system</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Poly Technologies showcases Silent Hunter - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>cheongwang-skylight</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Cheongwang (Skylight) Laser</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Cheongwang, Skylight, Block-I laser air-defense</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Hanwha Aerospace with ADD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>December 2024</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Initial operational fielding (Seoul area and frontline)</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>World's first laser weapon to reach operational military deployment; a 20kW fiber laser fully housed in a container-sized unit (~9m x 3m x 3m) with integrated radar mast, for point air-defense against small drones over Seoul.</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Army Recognition explicitly calls it container-sized.</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>https://armyrecognition.com/news/army-news/army-news-2024/south-korea-commissions-cheongwang-its-most-modern-laser-system-to-counter-aerial-threats</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>South Korea Commissions Cheongwang Laser - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/archives/archives-land-defense/land-defense-2024/south-korea-deploys-skylight-laser-weapon-to-protect-seoul-capital-and-frontline-areas-from-north-korean-drones</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>South Korea deploys Skylight laser - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>kawasaki-hel</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Kawasaki 100kW Laser C-UAS</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>KHI Electric-Drive High-Power Laser System</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Kawasaki Heavy Industries (KHI)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Installed aboard JMSDF test ship JS Asuka</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>100kW-class laser (ten fused 10kW fiber lasers) for counter-UAS, packaged into two 40-ft ISO container modules with a domed turret, installed on JS Asuka's deck for maritime trials.</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Prototype delivered to Japan MoD Feb 2023.</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2025/12/high-energy-laser-system-spotted-aboard-jmsdf-test-ship/</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>High-Energy Laser Aboard JMSDF Test Ship - Naval News</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>https://www.janes.com/osint-insights/defence-news/industry/dsei-japan-2023-kawasaki-heavy-industries-unveils-high-energy-laser-c-uas</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>KHI unveils high-energy laser C-UAS - Janes</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>edge-skyshield</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>EDGE SKYSHIELD</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SKYSHIELD, SKYSHIELD-TM C-UAS</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SIGN4L (EDGE Group)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2023-02-20</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>February 2023</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Unveiled at IDEX 2023</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Air defense / C-UAS</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>A multi-layered C-UAS solution (3D radar, EO/IR, RF direction-finders, jammers) networked into a unified C2 system, housed in a shock-proof, sealed container/cabinet for fixed or rapidly-deployable use; UAE MoD contract announced ~2024.</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Sources describe a compact shock-proof container/cabinet rather than confirmed full ISO dimensions.</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>IDEX 2023: EDGE launches SKYSHIELD C-UAS - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>https://www.sign4l.ae/</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SKYSHIELD Counter-UAS - SIGN4L</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>knds-drone-container</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>KNDS Containerized Drone Launcher</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>KNDS drone launch container, Helsing HX-2 / Tytan TI-1 METIS container</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>KNDS (France/Germany) with Helsing and Tytan</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>France / Germany</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Demonstrator unveiled at Eurosatory 2026</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Loitering munition</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>A self-contained 20-ft ISO container with independent power, environmental control and networking, housing dozens to 100+ effectors combining Helsing HX-2 strike drones and Tytan TI-1 METIS hard-kill interceptor drones; pitched as a response to Ukraine's Operation Spiderweb.</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Mock-up demonstrator/concept, not yet fielded; dual strike + interceptor role.</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>KNDS unveils containerized drone launcher concept - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>https://www.euro-sd.com/</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>KNDS showcases C-UAV capabilities at Eurosatory 2026 - ESD</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>destinus-hornet-b1</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Destinus Hornet Block 1 Containerized Interceptor</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Hornet B1, Destinus containerized interceptor drone launcher</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Destinus</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Switzerland (tested by Spain)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Test-fired aboard frigate Santa Maria and in land container config</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Air defense / C-UAS</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Canister-launched hard-kill interceptor drone engaging subsonic UAVs/swarms, fired from a modular containerized launch unit demonstrated on both a ship's deck and a land container configuration.</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Clearest verified containerized interceptor-drone launcher found.</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Spanish Navy Tests Hornet Block 1 from Santa Maria Frigate - Naval News</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>https://thedefensepost.com/</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Spanish Army Tests Destinus Hornet B1 in Container Launch Config - The Defense Post</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>roketsan-kara-atmaca</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roketsan Kara Atmaca Container Launcher</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Kara Atmaca, ATMACA-UM Container Launch System</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Roketsan</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Unveiled at IDEF 2025 (Istanbul)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Covert strike</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>A launcher disguised as an ordinary 20/40-ft commercial container, firing up to six Kara Atmaca land-attack/anti-ship cruise missiles (~250-280 km, 220kg warhead), movable by truck, rail or civilian cargo vessel.</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Roketsan states it is fully operational; multiple independent outlets confirm the container form factor.</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/army-news/2025/tuerkiye-debuts-kara-atmaca-container-launcher-at-idef-2025-for-covert-and-mobile-land-based-strike-roles</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Turkiye Debuts Kara Atmaca Container Launcher at IDEF 2025 - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>https://interestingengineering.com/military/shipping-containers-into-surprise-missile-launchers</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Turkey turns cargo container into missile-in-a-box - Interesting Engineering</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr"/>
+      <c r="W52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>roketsan-eren</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Roketsan EREN Containerized Loitering Munition Launcher</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>EREN Container Launch System, Roketsan EREN ground launcher</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Roketsan</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2025-07-22</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Unveiled at IDEF 2025 (Istanbul)</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Loitering munition</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>A truck-mounted launcher disguised as a civilian freight container, concealing up to 12 EREN jet-powered dual-role (anti-air/anti-ground) loitering munitions (35kg, &gt;100 km); serial production planned for 2026.</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Multiple independent outlets confirm the container disguise and IDEF 2025 debut.</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/archives/archives-land-defense/defense-news-army-2025/roketsan-debuts-containerized-eren-loitering-munition-launcher-at-idef-2025-for-covert-deep-strikes</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Roketsan Debuts Containerized EREN Launcher at IDEF 2025 - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>https://united24media.com/latest-news/inspired-by-ukraines-operation-spiderweb-turkey-unveils-hidden-drone-launcher-for-deep-strikes-10361</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Turkey Unveils Hidden Drone Launcher for Deep Strikes - United24</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr"/>
+      <c r="W53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>elbit-skystriker-container</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Elbit SkyStriker Containerized Launcher</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SkyStriker container launch configuration</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Elbit Systems</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2022-06-15</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Container launch configuration publicized (approximate)</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Loitering munition</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Electrically powered canister-launched loitering munition (up to 100 km, 10kg warhead); Elbit markets a container launch configuration packing 6 SkyStriker rounds per container for land or naval deployment.</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Container figure from Elbit product literature rather than a dedicated show unveiling; reveal date approximate.</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>https://www.elbitsystems.com/sites/default/files/2025-02/skystriker.pdf</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Elbit SkyStriker datasheet</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>https://www.battlepolicy.com/skystriker/</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>SkyStriker Israel's electric loitering munition - Battle Policy</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>elbit-trigon</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Elbit TRIGON Sea-to-Shore Weapon System</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>TRIGON naval rocket and missile launcher</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Elbit Systems</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2017-06-15</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Earliest trade-press coverage (approximate)</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Naval arsenal</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Modular deck launcher</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>A fixed-elevation deck-mounted launcher carrying two pods of four EXTRA guided rockets (150 km) each, installable permanently or as an add-on mission module above or below deck on small-to-medium naval craft.</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Elbit describes it as a bolt-on deck mission module rather than an explicit ISO container; container claim less firmly documented.</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>https://elbitsystems.com/product/trigon/</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>TRIGON Sea-to-Shore Weapon System - Elbit</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>https://www.asianmilitaryreview.com/2017/06/imi-systems-solutions-extend-modern-naval-capabilities/</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>IMI Systems naval solutions - Asian Military Review</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>northrop-ares</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Northrop Grumman AReS</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AReS, Advanced Reactive Strike, containerized ground-launched AARGM-ER</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Northrop Grumman</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2025-01-14</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>January 2025</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Unveiled at Surface Navy Association Symposium</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Strike missile</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>A 20/40-ft ISO container concealing a four-cell vertical launcher for ground-launched AARGM-ER anti-radiation missiles (~150 km), aimed at rapidly deployable suppression of enemy radar and air-defense sites.</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Northrop and Hanwha signed an MOA (Apr 2026) to co-develop an AReS rocket booster.</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/army-news/2025/new-northrop-grumman-ares-missile-launcher-enables-fast-deployment-against-enemy-radar</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>New Northrop Grumman AReS missile launcher - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>https://www.fw-mag.com/shownews/351/sna-2025-sees-northrop-grumman-push-ares-a-containerized-ground-launched-aargm-er</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>SNA 2025: Northrop Grumman push AReS - FW-MAG</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ruta-block-3</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Rheinmetall Destinus Ruta Block 3</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Ruta Block 3, RUTA Block III deep-strike cruise missile</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Rheinmetall Destinus Strike Systems</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Germany / Switzerland-Spain</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Unveiled at Eurosatory 2026</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Strike missile</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>A strategic deep-strike cruise missile (&gt;2,000 km, 250 kg warhead) launched exclusively from standard ISO shipping containers on vehicle (Rheinmetall HX truck) or maritime platforms, reaching firing readiness in ~2 minutes.</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Flight testing not scheduled until 2027; 100% European value chain targeted.</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>https://defence-industry.eu/rheinmetall-destinus-strike-systems-outlines-european-cruise-missile-priorities-with-ruta-block-3-and-initial-production/</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Rheinmetall Destinus Ruta Block 3 priorities - Defence Industry Europe</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>https://www.army-technology.com/news/rheinmetall-destinus-cruise-missile/</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Rheinmetall, Destinus 2,000km cruise missile - Army Technology</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr"/>
+      <c r="W57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>cm-401</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>CM-401 Containerized Deck Launcher</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CM-401 anti-ship ballistic missile, CASIC CM-401 deck launcher</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>CASIC (China Aerospace Science &amp; Industry Corp)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2018-11-06</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>November 2018</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Unveiled at Zhuhai Airshow China 2018</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Missile launcher</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Supersonic (Mach 4-6) anti-ship ballistic missile offered in a container-form deck launcher for surface ships (as well as an 8x8 truck TEL); pitched from 2025 for export coastal-defence use.</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Rebranded in army livery for coastal-defence export at IndoDefence 2025.</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>https://www.twz.com/24699/china-reveals-short-range-anti-ship-ballistic-missile-designed-to-dodge-enemy-defenses</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>China Reveals Short-Range Anti-Ship Ballistic Missile - TWZ</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>https://armyrecognition.com/news/army-news/2025/indodefence-2025-china-promotes-cm-401-anti-ship-missile-as-coastal-defense-for-foreign-customers</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>IndoDefence 2025: China promotes CM-401 as coastal defense - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>saab-rbs15-cdms</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Saab Coastal Defence Missile System (RBS15 CDMS)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Saab CDMS, RBS15 containerized coastal launcher</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Saab</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Publicly unveiled; on order for Swedish Armed Forces</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Artillery / coastal</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>A truck-carried launcher matching the footprint of a 20-ft ISO container, holding four RBS15 Mk3/Mk4 anti-ship missiles (&gt;300 km) with a shoot-and-scoot relocation under 120 seconds.</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>RBS15 fielded across Sweden, Finland, Germany, Poland, Bulgaria, Croatia.</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>https://www.saab.com/newsroom/stories/2025/september/a-powerful-new-deterrent-to-seaborne-threats</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>A powerful new deterrent to seaborne threats - Saab</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/navy-news/2025/saabs-new-coastal-defense-system-built-on-rbs15-missile-targets-growing-maritime-threats</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Saab's New Coastal Defense System - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr"/>
+      <c r="W59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>iris-t-slm-container</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Diehl IRIS-T SLM Containerized Fire Unit</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>IRIS-T SLM, IRIS-T SL container launcher/radar/TOC</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Diehl Defence</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2024-06-15</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>First fire unit delivered to German Armed Forces</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Air defense / C-UAS</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>IRIS-T SLM fire units (launcher, TRML-4D radar and IBMS tactical operations centre) are each built on standardised 20-ft ISO container frames for road/rail/sea/air transport; unmanned launchers reach readiness in 10 minutes.</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>Widely fielded to Ukraine and the Bundeswehr; container-frame design confirmed by multiple sources.</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>https://defence-industry.eu/diehl-defence-delivers-first-unit-of-iris-t-slm-system-to-german-armed-forces/</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Diehl delivers first IRIS-T SLM unit to German Armed Forces - Defence Industry Europe</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/archives/archives-land-defense/land-defense-2024/diehl-defence-delivers-first-iris-t-slm-air-defense-system-to-german-army</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Diehl delivers first IRIS-T SLM to German Army - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr"/>
+      <c r="W60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>boeing-clws</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Boeing Compact Laser Weapon System (containerized)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>CLWS, Boeing containerized laser weapon</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2024-06-01</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>June 2024</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Demonstrated in containerized config at Canada's IDEaS C-UAS Sandbox</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Directed energy</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>A fixed containerized configuration of Boeing's 5kW-class Compact Laser Weapon System, paired with radar cueing to detect, track and defeat FPV drones, mortar rounds and a five-UAS swarm at 200m-2.5km in Canadian trials.</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Tested alongside a Polaris RZR-mounted CLWS unit; hosted by DRDC at CFB Suffield.</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>https://www.boeing.com/features/2024/06/boeings-compact-lasers-shine-at-counter-drone-competition</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Boeing's compact lasers at counter-drone competition - Boeing</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>https://www.unmannedairspace.info/counter-uas-systems-and-policies/boeings-compact-laser-weapon-system-features-in-canadas-ideas-c-uas-trials/</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Boeing CLWS in Canada's IDEaS C-UAS trials - Unmanned Airspace</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>navypods-strike</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Royal Navy NavyPODS (Strike POD)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>PODS, Persistent Operational Deployment System, Strike POD</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>G3 Systems / QinetiQ for Royal Navy</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2021-09-14</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>September 2021</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Concept unveiled at DSEI 2021</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Modular system</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>A 20-ft ISO container-footprint modular payload system for RN vessels; the Strike POD variant hosts launchers for armed UAVs or loitering munitions plus a mission-planning area, part of an 18+ POD family.</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>Armed Strike POD remains a low-TRL demonstrator; G3 Systems selected as preferred supplier Nov 2025.</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>https://www.navylookout.com/thinking-inside-the-box-the-royal-navys-containerised-capability-concept/</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Royal Navy's containerised capability concept - Navy Lookout</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2025/11/g3-systems-selected-as-the-preferred-supplier-to-upgrade-navypods-capability/</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>G3 Systems preferred supplier for NavyPODS - Naval News</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>elbit-seagull-usv</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Elbit Seagull USV</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Seagull MCM/ASW USV, Seagull Mk3</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Elbit Systems</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2025-02-17</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>February 2025</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>4th-gen Seagull showcased at NAVDEX 2025</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Autonomous vehicle</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>A 12m multi-mission unmanned surface vessel (MCM/ASW/EW) that ships and deploys from a standard 40-ft ISO container; the planned 20m Mk3 adds deck space for a standardised 20-ft ISO container payload.</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>100% success in Royal Navy WISEX mine-hunting trials.</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>https://www.elbitsystems.com/unmanned/maritime/unmanned-surface-vessel/seagull-usv</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Seagull USV - Elbit Systems</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>https://www.janes.com/osint-insights/defence-news/sea/navdex-2025-elbit-system-showcases-fourth-generation-seagull-usv</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>NAVDEX 2025: 4th-gen Seagull USV - Janes</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>blacksea-chaser-usv</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BlackSea Technologies Chaser USV</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Chaser, GARC Block II</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>BlackSea Technologies</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Unveiled at Sea-Air-Space 2026</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Autonomous vehicle</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>A modular unmanned surface vessel engineered to fit inside and deploy from a standard 20-ft ISO container per a US Navy transportability requirement; carries JAGM launchers and EO/radar sensors.</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Built on ~5,000 operational hours of the earlier GARC design; unveiled alongside the larger Comet USV.</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2026/05/video-new-comet-and-chaser-usv-by-blacksea-technologies/</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>New Comet and Chaser USV by BlackSea Technologies - Naval News</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>https://www.blacksea.tech/chaser</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Chaser - BlackSea Technologies</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>speartooth-luuv</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>C2 Robotics Speartooth LUUV</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Speartooth, C2 Robotics long-range LUUV</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>C2 Robotics</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>First unit delivered to US Navy</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Autonomous vehicle</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>A long-range (2,000 km), 2,000m-depth large uncrewed undersea vehicle purpose-built to ship inside and deploy from a standard container via ramp or austere coastal infrastructure, without dedicated submarine support; ISR, mine warfare and strike delivery.</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Follows a 2025 NUWC Newport order for three long-range LUUVs.</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/navy-news/2026/us-navy-receives-first-australian-speartooth-luuv-drone-for-autonomous-underwater-strikes</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>US Navy receives first Australian Speartooth LUUV - Army Recognition</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>https://www.navaltoday.com/2026/05/05/australian-firm-commissions-first-us-export-luuv/</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Australian firm commissions first US export LUUV - Naval Today</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr"/>
+      <c r="W65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>xv-excalibur</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>XV Excalibur XLUUV</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Project Cetus XLUUV, Excalibur</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>MSubs Ltd / UK Submarine Delivery Agency</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Handed over to Royal Navy</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Autonomous vehicle</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>A 12m, ~19-25 tonne extra-large uncrewed underwater vehicle technology testbed, sized to be transported worldwide inside a standard 40-ft shipping container; controlled submerged from a remote centre in Australia during Talisman Sabre 2025.</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>Culmination of Project Cetus; payload bay can carry mines, smaller UUVs, sensors.</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2026/01/autonomous-submarine-xv-excalibur-handed-to-royal-navy/</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Autonomous submarine XV Excalibur handed to Royal Navy - Naval News</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>https://www.naval-technology.com/news/royal-navy-name-project-cetus-xluuv-excalibur/</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Royal Navy name Project Cetus XLUUV Excalibur - Naval Technology</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr"/>
+      <c r="W66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>bluewhale-uuv</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>IAI/tkMS BlueWhale UUV</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>BlueWhale AUV/XLUUV</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Israel Aerospace Industries / thyssenkrupp Marine Systems</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Israel / Germany</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>February 2026</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Delivered to German Navy at Eckernforde</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Autonomous vehicle</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>A 10.9m, 5.5-tonne autonomous underwater vehicle for ASW support, minehunting and covert ISR, engineered to be transported inside a standard 40-ft shipping container for deployment by land, air or sea; 10-30 day endurance to 300m depth.</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>Delivered under Germany's Kurs Marine 2035+ program after a 2-week German Navy trial.</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>https://www.tkmsgroup.com/news/article/autonomous-underwater-vehicle-bluewhale-handed-over-to-german-navy-delivery-by-tkms-and-israel-aerospace-industries-as-part-of-the-kurs-marine-2035-program</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>BlueWhale AUV handed over to German Navy - TKMS Group</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>https://www.armyrecognition.com/news/navy-news/2026/germanys-new-bluewhale-autonomous-underwater-vehicle-is-transforming-baltic-maritime-surveillance</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Germany's BlueWhale AUV - Army Recognition</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr"/>
+      <c r="W67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>anduril-slb-500m</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Anduril Surface-Launched Barracuda-500M</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SLB-500M, Surface-Launched Barracuda</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Anduril Industries</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Production agreement announcement</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Strike missile</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>A surface-launched Barracuda-500M variant paired with a standard 20-ft ISO launcher that can carry up to 16 rounds, for dispersed land and maritime strike; announced under the US Low-Cost Containerized Munitions effort.</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>From ChatGPT deep-research set; corroborated by Anduril and Naval News.</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>https://www.anduril.com/news/anduril-department-of-war-sign-production-agreement-for-surface-launched-barracuda-500m</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Anduril-DoW Production Agreement for SLB-500M - Anduril</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>https://www.navalnews.com/naval-news/2026/05/massive-u-s-missile-order-may-expand-american-anti-ship-arsenal/</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Massive US Missile Order May Expand Anti-Ship Arsenal - Naval News</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr"/>
+      <c r="W68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>iai-diamond</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>IAI DIAMOND Distributed Warfare System</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>DIAMOND, Distributed Warfare Solution</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Israel Aerospace Industries</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Official unveiling</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Modular system</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Modular deck launcher</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>A distributed-warfare architecture using container-footprint payload modules for ships and other platforms, able to host loitering munitions, Blue Spear, LORA, Barak MX and counter-UAS payloads in reconfigurable packages.</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>From ChatGPT deep-research set. Architecture/family rather than a fixed single-munition launcher.</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>https://www.iai.co.il/press/iai-unveils-diamond</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>IAI Unveils DIAMOND: New Distributed Warfare Solution - IAI</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>https://www.iai.co.il/product/diamond</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>DIAMOND - IAI</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr"/>
+      <c r="W69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>vampire-casket</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>L3Harris VAMPIRE CASKET</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>VAMPIRE CASKET, Containerized VAMPIRE counter-drone</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>L3Harris Technologies</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2025-10-09</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>October 2025</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Shown in L3Harris roadmap imagery</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Air defense / C-UAS</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Container form-factor</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>A standard-container mounting of L3Harris's VAMPIRE counter-drone system, combining its sensor-and-launcher architecture with kinetic effectors including laser-guided 70mm rockets.</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>From ChatGPT deep-research set. Depicted as a proposed family variant; dimensions/procurement/fielding limited.</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>https://www.twz.com/air/entire-family-of-vampire-counter-drone-systems-unveiled</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Entire Family Of VAMPIRE Counter-Drone Systems Unveiled - TWZ</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="inlineStr"/>
+      <c r="W70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Swap Destinus Hornet Block 1 photo (Spanish Navy frigate trial)
Replace images/destinus-hornet-b1.jpg with the DroneFirms hero image of the
Hornet Block 1 interceptor during its Spanish Navy frigate trial; update
photo credit/license/source.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XehwYvE8om8sW3on1oyWXA
</commit_message>
<xml_diff>
--- a/data/systems.xlsx
+++ b/data/systems.xlsx
@@ -669,17 +669,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Artvill / Wikimedia Commons</t>
+          <t>Destinus (via DroneFirms)</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>wikimedia</t>
+          <t>news</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>https://commons.wikimedia.org/wiki/File:Destinus_Hornet_au_Salon_du_Bourget_2025_1.jpg</t>
+          <t>https://media.dronefirms.com/articles/2026/img/destinus-hornet-block1-spanish-navy-frigate.jpg</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -6059,8 +6059,6 @@
           <t>Ivan Papanin begins sea trials with Kalibr - Army Recognition</t>
         </is>
       </c>
-      <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">

</xml_diff>

<commit_message>
Update KNDS entry photo to Eurosatory 2026 container shot, credit Army Recognition
Replace the KNDS containerized drone launcher image with the Eurosatory
2026 photo showing the deployed launcher and drone crate, and update the
photo credit/source to Army Recognition (@ArmyRecognition).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYo5Q3wp6WppK7FjE66P1M
</commit_message>
<xml_diff>
--- a/data/systems.xlsx
+++ b/data/systems.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="systems" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="systems" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -883,17 +883,17 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>KNDS Group</t>
+          <t>Army Recognition (@ArmyRecognition)</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>manufacturer</t>
+          <t>editorial</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>https://knds.com/en/press-releases/bolstering-mission-solution-portfolio-knds-showcases-first-drone-launch-container-prototype-at-eurosatory-2026-1</t>
+          <t>https://x.com/ArmyRecognition/status/2067157227341811904</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">

</xml_diff>